<commit_message>
New feature - Machine Status
</commit_message>
<xml_diff>
--- a/Data/Inputs/FilesTemplates/Template_Report.xlsx
+++ b/Data/Inputs/FilesTemplates/Template_Report.xlsx
@@ -1,29 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LuisRamos\OneDrive - Roboyo Global\Documents\UiPath\Personal\BotMonitor\Data\Inputs\FilesTemplates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10D6ABC2-1173-4033-947C-7F48DDA74B8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D7574BB-924C-4F56-B57A-63D6CC11B52A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="17496" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-30828" yWindow="-108" windowWidth="30936" windowHeight="17496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="2" r:id="rId1"/>
-    <sheet name="Jobs" sheetId="5" r:id="rId2"/>
-    <sheet name="Queues" sheetId="7" r:id="rId3"/>
-    <sheet name="Transactions" sheetId="6" r:id="rId4"/>
+    <sheet name="Machines" sheetId="9" r:id="rId2"/>
+    <sheet name="Jobs" sheetId="11" r:id="rId3"/>
+    <sheet name="Queues" sheetId="7" r:id="rId4"/>
+    <sheet name="Transactions" sheetId="6" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="28">
   <si>
     <t>Folder</t>
   </si>
@@ -98,6 +99,15 @@
   </si>
   <si>
     <t>Killed</t>
+  </si>
+  <si>
+    <t>Machine</t>
+  </si>
+  <si>
+    <t>RuntimeType</t>
+  </si>
+  <si>
+    <t>Runtimes</t>
   </si>
 </sst>
 </file>
@@ -139,7 +149,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -160,12 +170,6 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -180,7 +184,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FF9107EF-EA67-44EE-9EDB-7B3517B21E6D}" name="Folders" displayName="Folders" ref="A1:H2" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FF9107EF-EA67-44EE-9EDB-7B3517B21E6D}" name="Summary" displayName="Summary" ref="A1:H2" totalsRowShown="0">
   <autoFilter ref="A1:H2" xr:uid="{FF9107EF-EA67-44EE-9EDB-7B3517B21E6D}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{BBC179BF-6FE0-4762-B4D6-472663462EF3}" name="Folder"/>
@@ -197,22 +201,35 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E636B4FE-FCC7-46AE-A508-6702D4DB95D4}" name="Jobs" displayName="Jobs" ref="A1:G2" totalsRowShown="0">
-  <autoFilter ref="A1:G2" xr:uid="{E636B4FE-FCC7-46AE-A508-6702D4DB95D4}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{C9D7FE29-0221-40AD-8F4B-E736A7198BBA}" name="Folder"/>
-    <tableColumn id="5" xr3:uid="{D7A623AE-2ADB-48D3-8375-2BCF8D2F542E}" name="Process Name"/>
-    <tableColumn id="4" xr3:uid="{89DC987D-80E6-410F-88E1-763F4D949606}" name="Status"/>
-    <tableColumn id="3" xr3:uid="{5AB3991A-5936-4AFF-8C04-986AA047C15D}" name="Started" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{17ADD2AC-EE76-41A6-833C-E16200D6758D}" name="Ended" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{C6DB0571-083C-4B2A-A19D-EC0B0600C75B}" name="Source"/>
-    <tableColumn id="7" xr3:uid="{B22DD4C7-E799-43FE-AAC1-1C31EAA96426}" name="Notes"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{6B51CC8E-5997-4A2E-8DE3-26D95DE1D44F}" name="Machines" displayName="Machines" ref="A1:D2" totalsRowShown="0">
+  <autoFilter ref="A1:D2" xr:uid="{FF9107EF-EA67-44EE-9EDB-7B3517B21E6D}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{8B5947BF-04C4-41AD-A355-ED6548F44646}" name="Machine"/>
+    <tableColumn id="3" xr3:uid="{EF97040B-0E93-451A-B5BD-B8A44AB14DCA}" name="RuntimeType"/>
+    <tableColumn id="2" xr3:uid="{56B5DA68-D5F2-44E3-ACB0-F7E9C07DDA04}" name="Runtimes"/>
+    <tableColumn id="5" xr3:uid="{B66A261D-DA80-402D-9DF2-B83B97667BA3}" name="Status"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{5CDD289F-C5F8-41F0-949B-0C4EDF1FA490}" name="Jobs" displayName="Jobs" ref="A1:G2" totalsRowShown="0">
+  <autoFilter ref="A1:G2" xr:uid="{5CDD289F-C5F8-41F0-949B-0C4EDF1FA490}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{E4918B9F-83D7-43C3-BC9A-8C7BCDCAEB01}" name="Folder"/>
+    <tableColumn id="3" xr3:uid="{F5A720FB-4AB3-4ECC-82F7-BDB7783641B5}" name="Process Name"/>
+    <tableColumn id="2" xr3:uid="{F31DEFBF-09AF-4B7B-8F28-FADD83610A21}" name="Status"/>
+    <tableColumn id="9" xr3:uid="{E2C0D10A-D050-44F8-A359-F71CCA2FC159}" name="Started"/>
+    <tableColumn id="8" xr3:uid="{37A91E79-C940-4D62-94FA-86C781A611CF}" name="Ended"/>
+    <tableColumn id="7" xr3:uid="{BEDB7193-3DFE-4519-86DD-9D3B4C2CCF1F}" name="Source"/>
+    <tableColumn id="6" xr3:uid="{BC41BAE8-3608-483C-A274-DFA19A62C63B}" name="Notes"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{2D849C52-C558-4760-9865-8390B46AFAE6}" name="Queues" displayName="Queues" ref="A1:I2" insertRow="1" totalsRowShown="0">
   <autoFilter ref="A1:I2" xr:uid="{2D849C52-C558-4760-9865-8390B46AFAE6}"/>
   <tableColumns count="9">
@@ -230,7 +247,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{ED764BB9-1BA1-4C59-B722-9852B881D48E}" name="Transactions" displayName="Transactions" ref="A1:I2" totalsRowShown="0">
   <autoFilter ref="A1:I2" xr:uid="{ED764BB9-1BA1-4C59-B722-9852B881D48E}"/>
   <tableColumns count="9">
@@ -581,44 +598,28 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB689CB7-45CF-4551-B896-168D8E717AF9}">
+  <dimension ref="A1:D1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="42.6640625" customWidth="1"/>
-    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="26.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="108" customWidth="1"/>
+    <col min="1" max="1" width="28.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="28.6640625" customWidth="1"/>
+    <col min="4" max="4" width="26.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="C1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
@@ -629,6 +630,51 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD45DA84-67F5-47DE-A17B-ABD785F9F61F}">
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="24.6640625" customWidth="1"/>
+    <col min="2" max="2" width="46.5546875" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" customWidth="1"/>
+    <col min="4" max="4" width="11.5546875" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" customWidth="1"/>
+    <col min="6" max="6" width="19.21875" customWidth="1"/>
+    <col min="7" max="7" width="50.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33498675-E6D3-47A1-90D2-E021AE14BE7C}">
   <dimension ref="A1:I1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -690,7 +736,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CADEFBE-750A-44B4-BBF7-BF12CD92A6E4}">
   <dimension ref="A1:I1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
Get Triggers feature added
</commit_message>
<xml_diff>
--- a/Data/Inputs/FilesTemplates/Template_Report.xlsx
+++ b/Data/Inputs/FilesTemplates/Template_Report.xlsx
@@ -8,23 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LuisRamos\OneDrive - Roboyo Global\Documents\UiPath\Personal\BotMonitor\Data\Inputs\FilesTemplates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE53A358-44E1-4D06-8296-594D8AE7D9A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F813417-FB39-4A85-97DE-86CBA7E9DFB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="2" r:id="rId1"/>
     <sheet name="Jobs" sheetId="11" r:id="rId2"/>
     <sheet name="Queues" sheetId="7" r:id="rId3"/>
     <sheet name="Transactions" sheetId="6" r:id="rId4"/>
-    <sheet name="Machines" sheetId="9" r:id="rId5"/>
+    <sheet name="Triggers" sheetId="12" r:id="rId5"/>
+    <sheet name="Machines" sheetId="9" r:id="rId6"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="36">
   <si>
     <t>Folder</t>
   </si>
@@ -108,6 +109,30 @@
   </si>
   <si>
     <t>Runtimes</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Enabled</t>
+  </si>
+  <si>
+    <t>Process</t>
+  </si>
+  <si>
+    <t>Job Priority</t>
+  </si>
+  <si>
+    <t>Expression</t>
+  </si>
+  <si>
+    <t>Comments</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Queue Attached</t>
   </si>
 </sst>
 </file>
@@ -253,6 +278,24 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{22522E64-53B4-431C-A081-0B8110966532}" name="Triggers" displayName="Triggers" ref="A1:I2" insertRow="1" totalsRowShown="0">
+  <autoFilter ref="A1:I2" xr:uid="{22522E64-53B4-431C-A081-0B8110966532}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{C1D5ADC6-A665-474F-80B5-ECAE28468558}" name="Folder"/>
+    <tableColumn id="2" xr3:uid="{89BFDF92-6BC9-4428-AE55-258978353C95}" name="Name"/>
+    <tableColumn id="3" xr3:uid="{CEE3CCC5-946E-4C87-996F-0099D31123B5}" name="Enabled"/>
+    <tableColumn id="4" xr3:uid="{CA399E80-AB67-4E4D-AE40-149578970723}" name="Process"/>
+    <tableColumn id="5" xr3:uid="{120C2FCD-BF6A-413C-A7FE-612130B82129}" name="Job Priority"/>
+    <tableColumn id="8" xr3:uid="{946AAAB2-8017-4A27-A0F8-F5D1296F7BA2}" name="Type"/>
+    <tableColumn id="10" xr3:uid="{9CA18ACA-FFA7-4DAB-968C-AAAC23CB7941}" name="Queue Attached"/>
+    <tableColumn id="6" xr3:uid="{61D0BCE4-7F25-40E1-9E82-413606EC387F}" name="Expression"/>
+    <tableColumn id="7" xr3:uid="{2DCB3B67-EC95-4F4A-96C3-157F5BE154EE}" name="Comments"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{6B51CC8E-5997-4A2E-8DE3-26D95DE1D44F}" name="Machines" displayName="Machines" ref="A1:D2" totalsRowShown="0">
   <autoFilter ref="A1:D2" xr:uid="{FF9107EF-EA67-44EE-9EDB-7B3517B21E6D}"/>
   <tableColumns count="4">
@@ -758,6 +801,57 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD7A25E6-44EA-423B-BF23-619905DFE10F}">
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="23.88671875" customWidth="1"/>
+    <col min="2" max="2" width="25.109375" customWidth="1"/>
+    <col min="3" max="3" width="14.21875" customWidth="1"/>
+    <col min="4" max="4" width="26.33203125" customWidth="1"/>
+    <col min="5" max="7" width="19.6640625" customWidth="1"/>
+    <col min="8" max="8" width="26.109375" customWidth="1"/>
+    <col min="9" max="9" width="23.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB689CB7-45CF-4551-B896-168D8E717AF9}">
   <dimension ref="A1:D1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>